<commit_message>
Flight schedule veranderd, constraint voor rho teogevoegd en exit taxiways verbeterd
</commit_message>
<xml_diff>
--- a/solution_output.xlsx
+++ b/solution_output.xlsx
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>20.48993774616611</v>
+        <v>20.48993774616972</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>39.92839916451885</v>
+        <v>39.92839946393951</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -480,7 +480,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>59.36686085929978</v>
+        <v>59.3668611805042</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -488,7 +488,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>72.32583533789148</v>
+        <v>72.3258356590959</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>78.8053224049745</v>
+        <v>78.80532289600524</v>
       </c>
     </row>
   </sheetData>
@@ -535,7 +535,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>830.4899376321046</v>
+        <v>830.4899377445145</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -543,7 +543,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>849.9283993499994</v>
+        <v>849.928399462402</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -551,7 +551,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>869.3668610678978</v>
+        <v>869.3668611802896</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -559,7 +559,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>882.3258355464932</v>
+        <v>882.3258356588813</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -567,7 +567,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>888.805322785789</v>
+        <v>888.8053228981771</v>
       </c>
     </row>
   </sheetData>
@@ -606,7 +606,7 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>51.47948723929585</v>
+        <v>51.47948723914999</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -614,7 +614,7 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>64.43846171788755</v>
+        <v>64.43846171761106</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -622,7 +622,7 @@
         <v>12</v>
       </c>
       <c r="B6">
-        <v>109.7948723929585</v>
+        <v>109.7948723925365</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -630,7 +630,7 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>129.233334110846</v>
+        <v>149.3668611819332</v>
       </c>
     </row>
   </sheetData>
@@ -661,519 +661,519 @@
         <v>9</v>
       </c>
       <c r="B3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>141.4794872385573</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>154.4384617177275</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>199.7948723926529</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>239.3668611810726</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>231.4794872385464</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>244.4384617177275</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>289.7948723926529</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>329.3668611819448</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>321.4794872382736</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>334.4384617176693</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>379.7948723925947</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>419.3668611810726</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>411.4794872384373</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>424.4384617177275</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>469.7948723926529</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>528.3668611810722</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>501.4794872386337</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>514.4384617177275</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>559.7948723926529</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>599.3668611811863</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>591.4794872383936</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>604.4384617177275</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>649.7948723926529</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>709.3668611811856</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>681.4794872384664</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>694.4384617177275</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>739.7948723926529</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>779.3668611812209</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>771.4794872386046</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>784.4384617177275</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>829.7948723926529</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>869.3668611814101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
         <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>96.47948723929585</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>109.4384617178875</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6">
-        <v>154.7948723929585</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>174.233334110846</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>186.4794872392958</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>199.4384617178875</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6">
-        <v>244.7948723929585</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>264.233334110846</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>276.4794872392958</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>289.4384617178875</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6">
-        <v>334.7948723929585</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>354.233334110846</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>366.4794872392958</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>379.4384617178875</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6">
-        <v>424.7948723929585</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>444.233334110846</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>456.4794872392958</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>469.4384617178875</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6">
-        <v>514.7948723929585</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>534.233334110846</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>546.4794872392958</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>559.4384617178875</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6">
-        <v>604.7948723929585</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>624.233334110846</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>636.4794872392958</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>649.4384617178875</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6">
-        <v>694.7948723929585</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>714.233334110846</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>726.4794872392958</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>739.4384617178875</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6">
-        <v>784.7948723929585</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>804.233334110846</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>110.4899376815229</v>
+        <v>110.489937746158</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1181,7 +1181,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>129.9283993583977</v>
+        <v>129.9283994640456</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1189,7 +1189,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>149.366860905473</v>
+        <v>149.3668611819332</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1197,7 +1197,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>162.3258353840647</v>
+        <v>162.3258356605248</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1205,7 +1205,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>168.8053226233606</v>
+        <v>168.8053228998207</v>
       </c>
     </row>
   </sheetData>
@@ -1236,7 +1236,7 @@
         <v>9</v>
       </c>
       <c r="B3">
-        <v>810</v>
+        <v>855</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1244,7 +1244,7 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>816.4794872392958</v>
+        <v>861.4794872391358</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1252,7 +1252,7 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>829.4384617179021</v>
+        <v>874.4384617177275</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1260,7 +1260,7 @@
         <v>12</v>
       </c>
       <c r="B6">
-        <v>874.7948723930167</v>
+        <v>919.7948723926238</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1268,7 +1268,7 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>894.2333341109043</v>
+        <v>939.2333341105114</v>
       </c>
     </row>
   </sheetData>
@@ -1307,7 +1307,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>200.4899377461679</v>
+        <v>200.4899377458785</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1315,7 +1315,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>219.9283993242298</v>
+        <v>219.9283994598627</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1323,7 +1323,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>239.3668610421173</v>
+        <v>239.3668611777503</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1331,7 +1331,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>252.325835520709</v>
+        <v>252.325835656342</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1339,7 +1339,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>258.8053222674043</v>
+        <v>258.8053228956378</v>
       </c>
     </row>
   </sheetData>
@@ -1394,7 +1394,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>329.3668611819558</v>
+        <v>329.3668611819448</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1402,7 +1402,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>342.3258356605511</v>
+        <v>342.3258356605365</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1410,7 +1410,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>348.8053228998469</v>
+        <v>348.8053228998324</v>
       </c>
     </row>
   </sheetData>
@@ -1449,7 +1449,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>380.4899377461697</v>
+        <v>380.4899377458783</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1457,7 +1457,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>399.9283994640464</v>
+        <v>399.9283994599355</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1465,7 +1465,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>419.3668611819303</v>
+        <v>419.366861177823</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1473,7 +1473,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>432.325835660522</v>
+        <v>432.3258356564147</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1481,7 +1481,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>438.805322899817</v>
+        <v>438.8053228957106</v>
       </c>
     </row>
   </sheetData>
@@ -1520,7 +1520,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>470.4899373473763</v>
+        <v>470.4899377458875</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1528,7 +1528,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>489.9283990652639</v>
+        <v>489.9283994599537</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1536,7 +1536,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>509.3668607831403</v>
+        <v>509.3668611778412</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1544,7 +1544,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>522.3258352420962</v>
+        <v>522.3258356564329</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1552,7 +1552,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>528.8053223443421</v>
+        <v>528.8053228957288</v>
       </c>
     </row>
   </sheetData>
@@ -1591,7 +1591,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>560.4899377461679</v>
+        <v>560.4899377458783</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1599,7 +1599,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>579.9283990635759</v>
+        <v>579.9283994607395</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1607,7 +1607,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>599.3668607814616</v>
+        <v>599.366861178627</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1615,7 +1615,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>612.3258352600533</v>
+        <v>612.3258356572187</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1623,7 +1623,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>618.8053223401948</v>
+        <v>618.8053228965146</v>
       </c>
     </row>
   </sheetData>
@@ -1662,7 +1662,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>650.4899375165623</v>
+        <v>650.4899377458781</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1670,7 +1670,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>669.9283992344281</v>
+        <v>669.9283994636453</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1678,7 +1678,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>689.3668609523156</v>
+        <v>689.3668611812036</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1686,7 +1686,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>702.3258354309073</v>
+        <v>702.3258356590331</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1694,7 +1694,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>708.8053226702032</v>
+        <v>708.8053228965546</v>
       </c>
     </row>
   </sheetData>
@@ -1733,7 +1733,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>740.4899377461697</v>
+        <v>740.4899377458779</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1741,7 +1741,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>759.9283994640573</v>
+        <v>759.9283994603902</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1749,7 +1749,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>779.3668611819448</v>
+        <v>779.3668611782778</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1757,7 +1757,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>792.3258356605365</v>
+        <v>792.3258356568695</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1765,7 +1765,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>798.8053228998324</v>
+        <v>798.8053228961653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>